<commit_message>
allow for linear combination
</commit_message>
<xml_diff>
--- a/tests/paths/res/submodel.xlsx
+++ b/tests/paths/res/submodel.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\laghida\Documents\Github\cassy\tests\paths\res\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{34CD66CD-CBAA-40D0-B797-E4786892D301}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{97BF0FA5-8959-4E2C-A18D-9F94EB5BAF5D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Reference Event Fatigue" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="63">
   <si>
     <t>General Parameter</t>
   </si>
@@ -208,6 +208,12 @@
   </si>
   <si>
     <t>Is Short Overstress</t>
+  </si>
+  <si>
+    <t>combination</t>
+  </si>
+  <si>
+    <t>2-1</t>
   </si>
 </sst>
 </file>
@@ -263,7 +269,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -307,6 +313,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -614,19 +623,19 @@
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:K13"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="35.28515625" style="13" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="35.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="54.28515625" style="14" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="35.28515625" style="14" bestFit="1" customWidth="1"/>
-    <col min="5" max="6" width="35.28515625" style="15" bestFit="1" customWidth="1"/>
-    <col min="7" max="8" width="35.28515625" style="14" bestFit="1" customWidth="1"/>
-    <col min="9" max="10" width="35.28515625" style="13" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="35.28515625" style="12" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="35.26953125" style="13" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="35.26953125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="54.26953125" style="14" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="35.26953125" style="14" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="35.26953125" style="15" bestFit="1" customWidth="1"/>
+    <col min="7" max="8" width="35.26953125" style="14" bestFit="1" customWidth="1"/>
+    <col min="9" max="10" width="35.26953125" style="13" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="35.26953125" style="12" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="6" t="s">
         <v>7</v>
       </c>
@@ -661,7 +670,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="2" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="9">
         <v>1</v>
       </c>
@@ -696,7 +705,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="9">
         <v>2</v>
       </c>
@@ -731,7 +740,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="9"/>
       <c r="C4" s="10"/>
       <c r="D4" s="10"/>
@@ -743,7 +752,7 @@
       <c r="J4" s="9"/>
       <c r="K4" s="9"/>
     </row>
-    <row r="5" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="9"/>
       <c r="C5" s="11"/>
       <c r="D5" s="10"/>
@@ -755,7 +764,7 @@
       <c r="J5" s="9"/>
       <c r="K5" s="9"/>
     </row>
-    <row r="6" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="9"/>
       <c r="C6" s="10"/>
       <c r="D6" s="10"/>
@@ -766,7 +775,7 @@
       <c r="I6" s="9"/>
       <c r="J6" s="9"/>
     </row>
-    <row r="7" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="9"/>
       <c r="C7" s="11"/>
       <c r="D7" s="10"/>
@@ -777,7 +786,7 @@
       <c r="I7" s="9"/>
       <c r="J7" s="9"/>
     </row>
-    <row r="8" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="9"/>
       <c r="C8" s="10"/>
       <c r="D8" s="10"/>
@@ -788,7 +797,7 @@
       <c r="I8" s="9"/>
       <c r="J8" s="9"/>
     </row>
-    <row r="9" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="9"/>
       <c r="C9" s="11"/>
       <c r="D9" s="10"/>
@@ -799,7 +808,7 @@
       <c r="I9" s="9"/>
       <c r="J9" s="9"/>
     </row>
-    <row r="10" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="9"/>
       <c r="C10" s="10"/>
       <c r="D10" s="10"/>
@@ -810,7 +819,7 @@
       <c r="I10" s="9"/>
       <c r="J10" s="9"/>
     </row>
-    <row r="11" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="9"/>
       <c r="C11" s="11"/>
       <c r="D11" s="10"/>
@@ -821,7 +830,7 @@
       <c r="I11" s="9"/>
       <c r="J11" s="9"/>
     </row>
-    <row r="12" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="9"/>
       <c r="C12" s="10"/>
       <c r="D12" s="10"/>
@@ -832,7 +841,7 @@
       <c r="I12" s="9"/>
       <c r="J12" s="9"/>
     </row>
-    <row r="13" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="9"/>
       <c r="C13" s="11"/>
       <c r="D13" s="10"/>
@@ -854,19 +863,19 @@
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:J5"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="13.5703125" style="2" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="19.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="69.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.85546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="18.7109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="18.85546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="8" width="13.5703125" bestFit="1" customWidth="1"/>
-    <col min="9" max="10" width="13.5703125" style="2" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.54296875" style="2" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.453125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="69.81640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.81640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="18.7265625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="18.81640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="8" width="13.54296875" bestFit="1" customWidth="1"/>
+    <col min="9" max="10" width="13.54296875" style="2" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
         <v>7</v>
       </c>
@@ -898,7 +907,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:10" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="3">
         <v>1</v>
       </c>
@@ -930,7 +939,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:10" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:10" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="3">
         <v>1</v>
       </c>
@@ -962,7 +971,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:10" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:10" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="3">
         <v>2</v>
       </c>
@@ -994,7 +1003,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:10" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:10" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="3">
         <v>2</v>
       </c>
@@ -1036,22 +1045,22 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:J6"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:J7"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="27.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17.5703125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="18.85546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.5703125" style="4" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="21.140625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11.42578125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="27.7109375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="17.28515625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="18.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="27.26953125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.54296875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="18.81640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.54296875" style="4" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="21.1796875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.453125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="27.7265625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="17.26953125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="18.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>15</v>
       </c>
@@ -1083,7 +1092,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:10" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>18</v>
       </c>
@@ -1112,7 +1121,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="3" spans="1:10" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:10" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>20</v>
       </c>
@@ -1141,7 +1150,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="4" spans="1:10" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:10" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>22</v>
       </c>
@@ -1173,7 +1182,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="5" spans="1:10" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:10" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>24</v>
       </c>
@@ -1205,7 +1214,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="6" spans="1:10" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:10" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>25</v>
       </c>
@@ -1234,6 +1243,35 @@
         <v>38</v>
       </c>
       <c r="J6" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>61</v>
+      </c>
+      <c r="B7" t="s">
+        <v>34</v>
+      </c>
+      <c r="C7" t="s">
+        <v>39</v>
+      </c>
+      <c r="D7" t="s">
+        <v>36</v>
+      </c>
+      <c r="E7" s="4">
+        <v>1</v>
+      </c>
+      <c r="G7" t="s">
+        <v>37</v>
+      </c>
+      <c r="H7" t="s">
+        <v>38</v>
+      </c>
+      <c r="I7" t="s">
+        <v>38</v>
+      </c>
+      <c r="J7" t="s">
         <v>37</v>
       </c>
     </row>
@@ -1247,15 +1285,15 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:C6"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:C8"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="27.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="27.7265625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="22" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17.28515625" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.26953125" style="2" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>15</v>
       </c>
@@ -1266,7 +1304,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>18</v>
       </c>
@@ -1277,7 +1315,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>20</v>
       </c>
@@ -1288,7 +1326,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>22</v>
       </c>
@@ -1299,7 +1337,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>24</v>
       </c>
@@ -1310,7 +1348,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>25</v>
       </c>
@@ -1320,6 +1358,20 @@
       <c r="C6" s="3">
         <v>3</v>
       </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>61</v>
+      </c>
+      <c r="B7" t="s">
+        <v>23</v>
+      </c>
+      <c r="C7" s="16" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="C8" s="16"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1332,15 +1384,15 @@
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:E3"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="13.5703125" style="2" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.28515625" bestFit="1" customWidth="1"/>
-    <col min="4" max="5" width="13.5703125" style="2" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.54296875" style="2" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.54296875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.26953125" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="13.54296875" style="2" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
         <v>7</v>
       </c>
@@ -1357,7 +1409,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="3">
         <v>1</v>
       </c>
@@ -1374,7 +1426,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="3">
         <v>2</v>
       </c>
@@ -1402,15 +1454,15 @@
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:G4"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="24.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="6" width="13.5703125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="21.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="24.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.453125" bestFit="1" customWidth="1"/>
+    <col min="3" max="6" width="13.54296875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="21.7265625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1425,7 +1477,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -1436,12 +1488,12 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="G3" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="G4" t="s">
         <v>4</v>
       </c>

</xml_diff>